<commit_message>
Scrub Syncfusion version from trial watermark license link
</commit_message>
<xml_diff>
--- a/src/StaticSettingsTests/OutputsTests.ExcelWithCsv.verified.xlsx
+++ b/src/StaticSettingsTests/OutputsTests.ExcelWithCsv.verified.xlsx
@@ -107,7 +107,7 @@
     <t>Formula</t>
   </si>
   <si>
-    <t>https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzUuMS4zOQ==</t>
+    <t>https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=DeterministicVersion</t>
   </si>
   <si>
     <r>
@@ -328,7 +328,7 @@
     <xdr:sp macro="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="0" name="TextBox 1">
-          <a:hlinkClick xmlns:p7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" p7:id="rId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzUuMS4zOQ=="/>
+          <a:hlinkClick xmlns:p7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" p7:id="rId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=DeterministicVersion"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
@@ -2926,7 +2926,7 @@
     <mergeCell ref="A1001:T1001"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A1001" r:id="DeterministicId2" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzUuMS4zOQ==" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
+    <hyperlink ref="A1001" r:id="DeterministicId2" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=DeterministicVersion" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
   </hyperlinks>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2958,7 +2958,7 @@
     <mergeCell ref="A10:S10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A10" r:id="DeterministicId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzUuMS4zOQ==" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
+    <hyperlink ref="A10" r:id="DeterministicId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=DeterministicVersion" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>

</xml_diff>